<commit_message>
fix the ordering of the locale keys
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/00-shared-layout.xlsx
+++ b/translations/welsh-translations/xlsx/00-shared-layout.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="89">
   <si>
     <t>Translator notes</t>
   </si>
@@ -55,34 +55,193 @@
     <t/>
   </si>
   <si>
-    <t>common.warningIconFallback</t>
-  </si>
-  <si>
-    <t>Warning</t>
-  </si>
-  <si>
-    <t>common.regulation43Text</t>
-  </si>
-  <si>
-    <t>regulation 43</t>
-  </si>
-  <si>
-    <t>common.continue</t>
-  </si>
-  <si>
-    <t>Continue</t>
-  </si>
-  <si>
-    <t>common.opensInNewTab</t>
-  </si>
-  <si>
-    <t>opens in new tab</t>
-  </si>
-  <si>
-    <t>common.errorSummary.title</t>
-  </si>
-  <si>
-    <t>There is a problem</t>
+    <t>common.nav.menu</t>
+  </si>
+  <si>
+    <t>Menu</t>
+  </si>
+  <si>
+    <t>Dewislen</t>
+  </si>
+  <si>
+    <t>common.nav.menuLabel</t>
+  </si>
+  <si>
+    <t>Show or hide menu</t>
+  </si>
+  <si>
+    <t>common.phaseBanner.lead</t>
+  </si>
+  <si>
+    <t>This is a new service - your</t>
+  </si>
+  <si>
+    <t>Mae hwn yn wasanaeth newydd – bydd eich</t>
+  </si>
+  <si>
+    <t>common.phaseBanner.feedbackLink</t>
+  </si>
+  <si>
+    <t>feedback</t>
+  </si>
+  <si>
+    <t>adborth</t>
+  </si>
+  <si>
+    <t>common.phaseBanner.leadAfterLink</t>
+  </si>
+  <si>
+    <t>will help us to improve it.</t>
+  </si>
+  <si>
+    <t>yn ein helpu i’w wella.</t>
+  </si>
+  <si>
+    <t>common.phaseBanner.tag</t>
+  </si>
+  <si>
+    <t>Beta</t>
+  </si>
+  <si>
+    <t>beta</t>
+  </si>
+  <si>
+    <t>common.phaseBanner.label</t>
+  </si>
+  <si>
+    <t>Beta banner</t>
+  </si>
+  <si>
+    <t>common.languageSwitcher.label</t>
+  </si>
+  <si>
+    <t>Language</t>
+  </si>
+  <si>
+    <t>common.languageSwitcher.english</t>
+  </si>
+  <si>
+    <t>common.languageSwitcher.welsh</t>
+  </si>
+  <si>
+    <t>Cymraeg</t>
+  </si>
+  <si>
+    <t>common.nav.back</t>
+  </si>
+  <si>
+    <t>Back</t>
+  </si>
+  <si>
+    <t>Yn ôl</t>
+  </si>
+  <si>
+    <t>common.footer.getHelp</t>
+  </si>
+  <si>
+    <t>Get help</t>
+  </si>
+  <si>
+    <t>Cael help</t>
+  </si>
+  <si>
+    <t>common.footer.email</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Ebost</t>
+  </si>
+  <si>
+    <t>common.footer.telephone</t>
+  </si>
+  <si>
+    <t>Telephone</t>
+  </si>
+  <si>
+    <t>Ffôn</t>
+  </si>
+  <si>
+    <t>common.footer.openingTime</t>
+  </si>
+  <si>
+    <t>Monday to Friday, 8am to 6pm</t>
+  </si>
+  <si>
+    <t>Dydd Llun i ddydd Gwener, 8am i 6pm</t>
+  </si>
+  <si>
+    <t>common.footer.supportLinks</t>
+  </si>
+  <si>
+    <t>Support links</t>
+  </si>
+  <si>
+    <t>Dolenni cymorth</t>
+  </si>
+  <si>
+    <t>common.footer.cookies</t>
+  </si>
+  <si>
+    <t>Cookies</t>
+  </si>
+  <si>
+    <t>Cwcis</t>
+  </si>
+  <si>
+    <t>common.footer.privacy</t>
+  </si>
+  <si>
+    <t>Privacy</t>
+  </si>
+  <si>
+    <t>Preifatrwydd</t>
+  </si>
+  <si>
+    <t>common.footer.accessibility</t>
+  </si>
+  <si>
+    <t>Accessibility statement</t>
+  </si>
+  <si>
+    <t>Datganiad hygyrchedd</t>
+  </si>
+  <si>
+    <t>common.footer.allContent</t>
+  </si>
+  <si>
+    <t>All content is available under the</t>
+  </si>
+  <si>
+    <t>Mae’r holl gynnwys ar gael dan y</t>
+  </si>
+  <si>
+    <t>common.footer.openGovernmentLicence</t>
+  </si>
+  <si>
+    <t>Open Government Licence v3.0</t>
+  </si>
+  <si>
+    <t>Drwydded Llywodraeth Agored, fersiwn 3.0</t>
+  </si>
+  <si>
+    <t>common.footer.exceptWhere</t>
+  </si>
+  <si>
+    <t>, except where otherwise stated</t>
+  </si>
+  <si>
+    <t>, oni nodir yn wahanol</t>
+  </si>
+  <si>
+    <t>common.footer.crownCopyright</t>
+  </si>
+  <si>
+    <t>© Crown copyright</t>
+  </si>
+  <si>
+    <t>© Hawlfraint y Goron</t>
   </si>
   <si>
     <t>common.nav.home</t>
@@ -94,30 +253,6 @@
     <t>Hafan</t>
   </si>
   <si>
-    <t>common.nav.back</t>
-  </si>
-  <si>
-    <t>Back</t>
-  </si>
-  <si>
-    <t>Yn ôl</t>
-  </si>
-  <si>
-    <t>common.nav.menu</t>
-  </si>
-  <si>
-    <t>Menu</t>
-  </si>
-  <si>
-    <t>Dewislen</t>
-  </si>
-  <si>
-    <t>common.nav.menuLabel</t>
-  </si>
-  <si>
-    <t>Show or hide menu</t>
-  </si>
-  <si>
     <t>common.nav.manageAccount</t>
   </si>
   <si>
@@ -143,171 +278,6 @@
   </si>
   <si>
     <t>Allgofnodi</t>
-  </si>
-  <si>
-    <t>common.phaseBanner.tag</t>
-  </si>
-  <si>
-    <t>Beta</t>
-  </si>
-  <si>
-    <t>beta</t>
-  </si>
-  <si>
-    <t>common.phaseBanner.label</t>
-  </si>
-  <si>
-    <t>Beta banner</t>
-  </si>
-  <si>
-    <t>common.phaseBanner.lead</t>
-  </si>
-  <si>
-    <t>This is a new service - your</t>
-  </si>
-  <si>
-    <t>Mae hwn yn wasanaeth newydd – bydd eich</t>
-  </si>
-  <si>
-    <t>common.phaseBanner.feedbackLink</t>
-  </si>
-  <si>
-    <t>feedback</t>
-  </si>
-  <si>
-    <t>adborth</t>
-  </si>
-  <si>
-    <t>common.phaseBanner.leadAfterLink</t>
-  </si>
-  <si>
-    <t>will help us to improve it.</t>
-  </si>
-  <si>
-    <t>yn ein helpu i’w wella.</t>
-  </si>
-  <si>
-    <t>common.languageSwitcher.label</t>
-  </si>
-  <si>
-    <t>Language</t>
-  </si>
-  <si>
-    <t>common.languageSwitcher.english</t>
-  </si>
-  <si>
-    <t>common.languageSwitcher.welsh</t>
-  </si>
-  <si>
-    <t>Cymraeg</t>
-  </si>
-  <si>
-    <t>common.footer.getHelp</t>
-  </si>
-  <si>
-    <t>Get help</t>
-  </si>
-  <si>
-    <t>Cael help</t>
-  </si>
-  <si>
-    <t>common.footer.email</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>Ebost</t>
-  </si>
-  <si>
-    <t>common.footer.telephone</t>
-  </si>
-  <si>
-    <t>Telephone</t>
-  </si>
-  <si>
-    <t>Ffôn</t>
-  </si>
-  <si>
-    <t>common.footer.openingTime</t>
-  </si>
-  <si>
-    <t>Monday to Friday, 8am to 6pm</t>
-  </si>
-  <si>
-    <t>Dydd Llun i ddydd Gwener, 8am i 6pm</t>
-  </si>
-  <si>
-    <t>common.footer.supportLinks</t>
-  </si>
-  <si>
-    <t>Support links</t>
-  </si>
-  <si>
-    <t>Dolenni cymorth</t>
-  </si>
-  <si>
-    <t>common.footer.cookies</t>
-  </si>
-  <si>
-    <t>Cookies</t>
-  </si>
-  <si>
-    <t>Cwcis</t>
-  </si>
-  <si>
-    <t>common.footer.privacy</t>
-  </si>
-  <si>
-    <t>Privacy</t>
-  </si>
-  <si>
-    <t>Preifatrwydd</t>
-  </si>
-  <si>
-    <t>common.footer.accessibility</t>
-  </si>
-  <si>
-    <t>Accessibility statement</t>
-  </si>
-  <si>
-    <t>Datganiad hygyrchedd</t>
-  </si>
-  <si>
-    <t>common.footer.allContent</t>
-  </si>
-  <si>
-    <t>All content is available under the</t>
-  </si>
-  <si>
-    <t>Mae’r holl gynnwys ar gael dan y</t>
-  </si>
-  <si>
-    <t>common.footer.openGovernmentLicence</t>
-  </si>
-  <si>
-    <t>Open Government Licence v3.0</t>
-  </si>
-  <si>
-    <t>Drwydded Llywodraeth Agored, fersiwn 3.0</t>
-  </si>
-  <si>
-    <t>common.footer.exceptWhere</t>
-  </si>
-  <si>
-    <t>, except where otherwise stated</t>
-  </si>
-  <si>
-    <t>, oni nodir yn wahanol</t>
-  </si>
-  <si>
-    <t>common.footer.crownCopyright</t>
-  </si>
-  <si>
-    <t>© Crown copyright</t>
-  </si>
-  <si>
-    <t>© Hawlfraint y Goron</t>
   </si>
 </sst>
 </file>
@@ -706,7 +676,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" hidden="1" customWidth="1"/>
@@ -784,7 +754,7 @@
         <v>15</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>13</v>
@@ -792,7 +762,7 @@
     </row>
     <row r="7" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>9</v>
@@ -801,7 +771,7 @@
         <v>10</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>13</v>
@@ -812,7 +782,7 @@
     </row>
     <row r="8" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>9</v>
@@ -821,10 +791,10 @@
         <v>10</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>13</v>
@@ -832,7 +802,7 @@
     </row>
     <row r="9" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>9</v>
@@ -841,10 +811,10 @@
         <v>10</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>13</v>
@@ -852,7 +822,7 @@
     </row>
     <row r="10" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>9</v>
@@ -861,10 +831,10 @@
         <v>10</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>13</v>
@@ -872,7 +842,7 @@
     </row>
     <row r="11" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>9</v>
@@ -881,10 +851,10 @@
         <v>10</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>13</v>
@@ -892,7 +862,7 @@
     </row>
     <row r="12" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>9</v>
@@ -901,10 +871,10 @@
         <v>10</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>13</v>
@@ -912,7 +882,7 @@
     </row>
     <row r="13" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>9</v>
@@ -921,10 +891,10 @@
         <v>10</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>13</v>
@@ -932,7 +902,7 @@
     </row>
     <row r="14" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>9</v>
@@ -941,7 +911,7 @@
         <v>10</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>13</v>
@@ -952,7 +922,7 @@
     </row>
     <row r="15" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>9</v>
@@ -961,10 +931,10 @@
         <v>10</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>13</v>
@@ -1044,7 +1014,7 @@
         <v>48</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>13</v>
+        <v>49</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>13</v>
@@ -1052,7 +1022,7 @@
     </row>
     <row r="20" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>9</v>
@@ -1061,10 +1031,10 @@
         <v>10</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>13</v>
@@ -1072,7 +1042,7 @@
     </row>
     <row r="21" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>9</v>
@@ -1081,10 +1051,10 @@
         <v>10</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>13</v>
@@ -1092,7 +1062,7 @@
     </row>
     <row r="22" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>9</v>
@@ -1101,10 +1071,10 @@
         <v>10</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>13</v>
@@ -1112,7 +1082,7 @@
     </row>
     <row r="23" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>9</v>
@@ -1121,10 +1091,10 @@
         <v>10</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>13</v>
+        <v>61</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>13</v>
@@ -1132,7 +1102,7 @@
     </row>
     <row r="24" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>9</v>
@@ -1141,10 +1111,10 @@
         <v>10</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>13</v>
+        <v>64</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>13</v>
@@ -1152,7 +1122,7 @@
     </row>
     <row r="25" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>9</v>
@@ -1161,10 +1131,10 @@
         <v>10</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>13</v>
+        <v>67</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>13</v>
@@ -1172,7 +1142,7 @@
     </row>
     <row r="26" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>9</v>
@@ -1181,10 +1151,10 @@
         <v>10</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>13</v>
@@ -1192,7 +1162,7 @@
     </row>
     <row r="27" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>9</v>
@@ -1201,10 +1171,10 @@
         <v>10</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>13</v>
@@ -1212,7 +1182,7 @@
     </row>
     <row r="28" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>9</v>
@@ -1221,10 +1191,10 @@
         <v>10</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>13</v>
@@ -1232,7 +1202,7 @@
     </row>
     <row r="29" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>9</v>
@@ -1241,10 +1211,10 @@
         <v>10</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>13</v>
@@ -1252,7 +1222,7 @@
     </row>
     <row r="30" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>9</v>
@@ -1261,10 +1231,10 @@
         <v>10</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>13</v>
@@ -1272,7 +1242,7 @@
     </row>
     <row r="31" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>9</v>
@@ -1281,10 +1251,10 @@
         <v>10</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>13</v>
@@ -1292,7 +1262,7 @@
     </row>
     <row r="32" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>9</v>
@@ -1301,117 +1271,17 @@
         <v>10</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="F32" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="33" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="34" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="35" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="36" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="F36" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="37" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="E37" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:F37"/>
+  <autoFilter ref="A4:F32"/>
   <mergeCells count="2">
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="D2:F2"/>

</xml_diff>

<commit_message>
MO-198 apply welsh translations
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/00-shared-layout.xlsx
+++ b/translations/welsh-translations/xlsx/00-shared-layout.xlsx
@@ -1,17 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8EAE257-5DF8-4F82-9548-1AFA6AD97DAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Welsh translations" state="visible" r:id="rId4"/>
+    <sheet name="Welsh translations" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="93">
   <si>
     <t>Translator notes</t>
   </si>
@@ -34,9 +38,6 @@
     <t>Welsh</t>
   </si>
   <si>
-    <t>Figma link</t>
-  </si>
-  <si>
     <t>common.serviceName</t>
   </si>
   <si>
@@ -49,9 +50,6 @@
     <t>Report packaging data</t>
   </si>
   <si>
-    <t>Rhoi gwybod am ddata pecynwaith</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
@@ -103,9 +101,6 @@
     <t>Beta</t>
   </si>
   <si>
-    <t>beta</t>
-  </si>
-  <si>
     <t>common.phaseBanner.label</t>
   </si>
   <si>
@@ -151,9 +146,6 @@
     <t>Email</t>
   </si>
   <si>
-    <t>Ebost</t>
-  </si>
-  <si>
     <t>common.footer.telephone</t>
   </si>
   <si>
@@ -259,9 +251,6 @@
     <t>Manage account</t>
   </si>
   <si>
-    <t>Rheoli’r Cyfrif</t>
-  </si>
-  <si>
     <t>common.nav.signIn</t>
   </si>
   <si>
@@ -278,27 +267,59 @@
   </si>
   <si>
     <t>Allgofnodi</t>
+  </si>
+  <si>
+    <t>Figma link for this content</t>
+  </si>
+  <si>
+    <t>There is no Figma link for this content.</t>
+  </si>
+  <si>
+    <t>Riportio data pecynwaith</t>
+  </si>
+  <si>
+    <t>Dangos neu guddio'r ddewislen</t>
+  </si>
+  <si>
+    <t>Baner beta</t>
+  </si>
+  <si>
+    <t>Iaith</t>
+  </si>
+  <si>
+    <t>Saesneg</t>
+  </si>
+  <si>
+    <t>E-bost</t>
+  </si>
+  <si>
+    <t>Rheoli’r cyfrif</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -326,15 +347,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -675,9 +699,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F32"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50" hidden="1" customWidth="1"/>
     <col min="2" max="3" width="35" hidden="1" customWidth="1"/>
@@ -685,608 +709,608 @@
     <col min="6" max="6" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="4:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="D1" s="2" t="s">
+    <row r="1" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-    </row>
-    <row r="2" ht="36" customHeight="1" spans="4:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="D2" s="1" t="s">
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+    </row>
+    <row r="2" spans="1:6" s="1" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-    </row>
-    <row r="3" ht="36" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="4" ht="24" customHeight="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+    </row>
+    <row r="3" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="1:6" s="2" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="B5" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>11</v>
-      </c>
       <c r="E5" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="B6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="6" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="1" t="s">
+      <c r="F6" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="B7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="E7" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" s="1" t="s">
+      <c r="B8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" s="1" t="s">
+      <c r="F8" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="B9" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="F8" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="E9" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" s="1" t="s">
+      <c r="F9" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="B10" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F9" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="E10" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10" s="1" t="s">
+      <c r="F10" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="B11" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F10" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="E11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" s="1" t="s">
+      <c r="B12" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E12" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F11" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="12" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="B13" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" s="1" t="s">
+      <c r="E13" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>35</v>
-      </c>
       <c r="B14" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>13</v>
+        <v>90</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B15" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D15" s="1" t="s">
+      <c r="E16" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E15" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+      <c r="F16" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D16" s="1" t="s">
+      <c r="B17" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="E17" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="F16" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="17" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+      <c r="F17" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D17" s="1" t="s">
+      <c r="B18" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="E18" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="F17" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
+      <c r="B19" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D18" s="1" t="s">
+      <c r="E19" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="F19" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="F18" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="19" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+      <c r="B20" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B19" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D19" s="1" t="s">
+      <c r="E20" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="F20" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="F19" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="20" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+      <c r="B21" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D20" s="1" t="s">
+      <c r="E21" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="F21" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F20" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="21" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+      <c r="B22" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B21" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D21" s="1" t="s">
+      <c r="E22" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="F22" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="F21" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="22" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
+      <c r="B23" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D23" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D22" s="1" t="s">
+      <c r="E23" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="F23" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F22" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="23" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
+      <c r="B24" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D24" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D23" s="1" t="s">
+      <c r="E24" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="F24" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="F23" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="24" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
+      <c r="B25" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D25" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D24" s="1" t="s">
+      <c r="E25" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="E24" s="1" t="s">
+      <c r="F25" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="F24" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="25" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
+      <c r="B26" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D26" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D25" s="1" t="s">
+      <c r="E26" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="E25" s="1" t="s">
+      <c r="F26" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="F25" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="26" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
+      <c r="B27" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D27" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D26" s="1" t="s">
+      <c r="E27" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="E26" s="1" t="s">
+      <c r="F27" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="F26" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="27" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
+      <c r="B28" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D28" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B27" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D27" s="1" t="s">
+      <c r="E28" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E27" s="1" t="s">
+      <c r="F28" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="F27" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="28" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
+      <c r="B29" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D29" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B28" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D28" s="1" t="s">
+      <c r="E29" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="E28" s="1" t="s">
+      <c r="F29" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="F28" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="29" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
+      <c r="B30" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D30" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B29" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D29" s="1" t="s">
+      <c r="E30" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="E29" s="1" t="s">
+      <c r="B31" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D31" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="F29" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="30" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
+      <c r="E31" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="B30" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D30" s="1" t="s">
+      <c r="F31" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E30" s="1" t="s">
+      <c r="B32" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D32" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="F30" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="31" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
+      <c r="E32" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B31" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="32" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>88</v>
-      </c>
       <c r="F32" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F32"/>
+  <autoFilter ref="A4:F32" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="2">
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="D2:F2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
MO-430 - renistate locales + translations - fixes en & cy locales JSON - regenerate translations
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/00-shared-layout.xlsx
+++ b/translations/welsh-translations/xlsx/00-shared-layout.xlsx
@@ -1,21 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8EAE257-5DF8-4F82-9548-1AFA6AD97DAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Welsh translations" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Welsh translations" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="92">
   <si>
     <t>Translator notes</t>
   </si>
@@ -38,6 +34,9 @@
     <t>Welsh</t>
   </si>
   <si>
+    <t>Figma link</t>
+  </si>
+  <si>
     <t>common.serviceName</t>
   </si>
   <si>
@@ -50,6 +49,9 @@
     <t>Report packaging data</t>
   </si>
   <si>
+    <t>Riportio data pecynwaith</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
@@ -68,6 +70,9 @@
     <t>Show or hide menu</t>
   </si>
   <si>
+    <t>Dangos neu guddio'r ddewislen</t>
+  </si>
+  <si>
     <t>common.phaseBanner.lead</t>
   </si>
   <si>
@@ -107,15 +112,24 @@
     <t>Beta banner</t>
   </si>
   <si>
+    <t>Baner beta</t>
+  </si>
+  <si>
     <t>common.languageSwitcher.label</t>
   </si>
   <si>
     <t>Language</t>
   </si>
   <si>
+    <t>Iaith</t>
+  </si>
+  <si>
     <t>common.languageSwitcher.english</t>
   </si>
   <si>
+    <t>Saesneg</t>
+  </si>
+  <si>
     <t>common.languageSwitcher.welsh</t>
   </si>
   <si>
@@ -146,6 +160,9 @@
     <t>Email</t>
   </si>
   <si>
+    <t>E-bost</t>
+  </si>
+  <si>
     <t>common.footer.telephone</t>
   </si>
   <si>
@@ -251,6 +268,9 @@
     <t>Manage account</t>
   </si>
   <si>
+    <t>Rheoli’r cyfrif</t>
+  </si>
+  <si>
     <t>common.nav.signIn</t>
   </si>
   <si>
@@ -267,59 +287,27 @@
   </si>
   <si>
     <t>Allgofnodi</t>
-  </si>
-  <si>
-    <t>Figma link for this content</t>
-  </si>
-  <si>
-    <t>There is no Figma link for this content.</t>
-  </si>
-  <si>
-    <t>Riportio data pecynwaith</t>
-  </si>
-  <si>
-    <t>Dangos neu guddio'r ddewislen</t>
-  </si>
-  <si>
-    <t>Baner beta</t>
-  </si>
-  <si>
-    <t>Iaith</t>
-  </si>
-  <si>
-    <t>Saesneg</t>
-  </si>
-  <si>
-    <t>E-bost</t>
-  </si>
-  <si>
-    <t>Rheoli’r cyfrif</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -347,18 +335,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -699,9 +684,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F32"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" hidden="1" customWidth="1"/>
     <col min="2" max="3" width="35" hidden="1" customWidth="1"/>
@@ -709,608 +694,608 @@
     <col min="6" max="6" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D1" s="3" t="s">
+    <row r="1" ht="24" customHeight="1" spans="4:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-    </row>
-    <row r="2" spans="1:6" s="1" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D2" s="4" t="s">
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" ht="36" customHeight="1" spans="4:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-    </row>
-    <row r="3" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="1:6" s="2" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" ht="36" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" ht="24" customHeight="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="2" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F4" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>86</v>
+        <v>12</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>87</v>
+        <v>19</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>88</v>
+        <v>33</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>89</v>
+        <v>36</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E14" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="31" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="32" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D32" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="F14" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E18" s="1" t="s">
+      <c r="E32" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="F18" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>83</v>
-      </c>
       <c r="F32" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F32" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A4:F32"/>
   <mergeCells count="2">
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="D2:F2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add new manage obligations page
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/00-shared-layout.xlsx
+++ b/translations/welsh-translations/xlsx/00-shared-layout.xlsx
@@ -1,21 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8EAE257-5DF8-4F82-9548-1AFA6AD97DAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Welsh translations" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Welsh translations" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="92">
   <si>
     <t>Translator notes</t>
   </si>
@@ -38,6 +34,9 @@
     <t>Welsh</t>
   </si>
   <si>
+    <t>Figma link</t>
+  </si>
+  <si>
     <t>common.serviceName</t>
   </si>
   <si>
@@ -50,6 +49,9 @@
     <t>Report packaging data</t>
   </si>
   <si>
+    <t>Riportio data pecynwaith</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
@@ -68,6 +70,9 @@
     <t>Show or hide menu</t>
   </si>
   <si>
+    <t>Dangos neu guddio'r ddewislen</t>
+  </si>
+  <si>
     <t>common.phaseBanner.lead</t>
   </si>
   <si>
@@ -107,15 +112,24 @@
     <t>Beta banner</t>
   </si>
   <si>
+    <t>Baner beta</t>
+  </si>
+  <si>
     <t>common.languageSwitcher.label</t>
   </si>
   <si>
     <t>Language</t>
   </si>
   <si>
+    <t>Iaith</t>
+  </si>
+  <si>
     <t>common.languageSwitcher.english</t>
   </si>
   <si>
+    <t>Saesneg</t>
+  </si>
+  <si>
     <t>common.languageSwitcher.welsh</t>
   </si>
   <si>
@@ -146,6 +160,9 @@
     <t>Email</t>
   </si>
   <si>
+    <t>E-bost</t>
+  </si>
+  <si>
     <t>common.footer.telephone</t>
   </si>
   <si>
@@ -251,6 +268,18 @@
     <t>Manage account</t>
   </si>
   <si>
+    <t>Rheoli’r cyfrif</t>
+  </si>
+  <si>
+    <t>common.nav.signOut</t>
+  </si>
+  <si>
+    <t>Sign out</t>
+  </si>
+  <si>
+    <t>Allgofnodi</t>
+  </si>
+  <si>
     <t>common.nav.signIn</t>
   </si>
   <si>
@@ -258,68 +287,27 @@
   </si>
   <si>
     <t>Mewngofnodi</t>
-  </si>
-  <si>
-    <t>common.nav.signOut</t>
-  </si>
-  <si>
-    <t>Sign out</t>
-  </si>
-  <si>
-    <t>Allgofnodi</t>
-  </si>
-  <si>
-    <t>Figma link for this content</t>
-  </si>
-  <si>
-    <t>There is no Figma link for this content.</t>
-  </si>
-  <si>
-    <t>Riportio data pecynwaith</t>
-  </si>
-  <si>
-    <t>Dangos neu guddio'r ddewislen</t>
-  </si>
-  <si>
-    <t>Baner beta</t>
-  </si>
-  <si>
-    <t>Iaith</t>
-  </si>
-  <si>
-    <t>Saesneg</t>
-  </si>
-  <si>
-    <t>E-bost</t>
-  </si>
-  <si>
-    <t>Rheoli’r cyfrif</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -347,18 +335,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -699,9 +684,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F32"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" hidden="1" customWidth="1"/>
     <col min="2" max="3" width="35" hidden="1" customWidth="1"/>
@@ -709,608 +694,608 @@
     <col min="6" max="6" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D1" s="3" t="s">
+    <row r="1" ht="24" customHeight="1" spans="4:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-    </row>
-    <row r="2" spans="1:6" s="1" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D2" s="4" t="s">
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" ht="36" customHeight="1" spans="4:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-    </row>
-    <row r="3" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="1:6" s="2" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" ht="36" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" ht="24" customHeight="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="2" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F4" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>86</v>
+        <v>12</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>87</v>
+        <v>19</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>88</v>
+        <v>33</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>89</v>
+        <v>36</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E14" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="31" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="32" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D32" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="F14" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E18" s="1" t="s">
+      <c r="E32" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="F18" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>83</v>
-      </c>
       <c r="F32" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F32" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A4:F32"/>
   <mergeCells count="2">
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="D2:F2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>